<commit_message>
Update command support spreadsheet
</commit_message>
<xml_diff>
--- a/Reports/Command Support.xlsx
+++ b/Reports/Command Support.xlsx
@@ -21765,7 +21765,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L171" s="34" t="n"/>
+      <c r="L171" s="34" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="M171" s="25" t="inlineStr">
         <is>
           <t>Pass</t>

</xml_diff>